<commit_message>
v1.2.2; updated internal Dependency document
</commit_message>
<xml_diff>
--- a/documentation/Dependencies.xlsx
+++ b/documentation/Dependencies.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ba4eb5\Desktop\Skalierung\Skalierungspaket\scaling\documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lifbide-my.sharepoint.com/personal/nu004438_lifbi_de/Documents/Desktop/NEPSroutines/Paket/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C9A063A-FB45-4A13-A925-35BE1998D4F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{2C9A063A-FB45-4A13-A925-35BE1998D4F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{019BBB59-B9A3-4A76-BC0E-B73DB9EBA4D0}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{73FFCF87-98C9-4C4C-9C88-8C4AFB5511E6}"/>
+    <workbookView xWindow="-28920" yWindow="6555" windowWidth="29040" windowHeight="17520" xr2:uid="{73FFCF87-98C9-4C4C-9C88-8C4AFB5511E6}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -276,7 +276,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -302,7 +302,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -713,28 +712,28 @@
       </c>
       <c r="O2" s="3"/>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3">
-        <v>1</v>
-      </c>
-      <c r="M4" s="3">
-        <v>1</v>
-      </c>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="Q4" t="s">
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5">
+        <v>1</v>
+      </c>
+      <c r="M4" s="5">
+        <v>1</v>
+      </c>
+      <c r="N4" s="5"/>
+      <c r="O4" s="5"/>
+      <c r="Q4" s="4" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1122,10 +1121,10 @@
       <c r="O20" s="3"/>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A22" s="13" t="s">
+      <c r="A22" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="13"/>
+      <c r="B22" s="1"/>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">

</xml_diff>